<commit_message>
bad commit - code is good but doesn't pass tests
</commit_message>
<xml_diff>
--- a/examples/example01/HFP_template.xlsx
+++ b/examples/example01/HFP_template.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,10 +479,15 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>HSA ctrb</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
@@ -504,8 +509,11 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -523,8 +531,11 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -542,8 +553,11 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -561,8 +575,11 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -580,8 +597,11 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -599,8 +619,11 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -618,8 +641,11 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -637,8 +663,11 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -656,8 +685,11 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -675,8 +707,11 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -694,8 +729,11 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -713,8 +751,11 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
       <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -732,8 +773,11 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -751,8 +795,11 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -770,8 +817,11 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
       <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -789,8 +839,11 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -808,8 +861,11 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
       <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -827,8 +883,11 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
       <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -846,8 +905,11 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
       <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -865,8 +927,11 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
       <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -884,8 +949,11 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
       <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -903,8 +971,11 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
       <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -922,8 +993,11 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
       <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -941,8 +1015,11 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
       <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -960,8 +1037,11 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
       <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -979,8 +1059,11 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
       <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -998,8 +1081,11 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
       <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1017,8 +1103,11 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
       <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1036,8 +1125,11 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
       <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1055,8 +1147,11 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
       <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1074,8 +1169,11 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
       <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1093,8 +1191,11 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
       <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1112,8 +1213,11 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
       <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1131,8 +1235,11 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
       <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1150,8 +1257,11 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
       <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1169,8 +1279,11 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
       <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1188,8 +1301,11 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
       <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1202,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1253,10 +1369,15 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>HSA ctrb</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Roth conv</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>big-ticket items</t>
         </is>
@@ -1278,8 +1399,11 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1297,8 +1421,11 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1316,8 +1443,11 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1335,8 +1465,11 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1354,8 +1487,11 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1373,8 +1509,11 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1392,8 +1531,11 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1411,8 +1553,11 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1430,8 +1575,11 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1449,8 +1597,11 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1468,8 +1619,11 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1487,8 +1641,11 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
       <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1506,8 +1663,11 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1525,8 +1685,11 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1544,8 +1707,11 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
       <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1563,8 +1729,11 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1582,8 +1751,11 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
       <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1601,8 +1773,11 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
       <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1620,8 +1795,11 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
       <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1639,8 +1817,11 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
       <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1658,8 +1839,11 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
       <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1677,8 +1861,11 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
       <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1696,8 +1883,11 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
       <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1715,8 +1905,11 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
       <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1734,8 +1927,11 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
       <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1753,8 +1949,11 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
       <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1772,8 +1971,11 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
       <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1791,8 +1993,11 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
       <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1810,8 +2015,11 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
       <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1829,8 +2037,11 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
       <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1848,8 +2059,11 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
       <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1867,8 +2081,11 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
       <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1886,8 +2103,11 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
       <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1905,8 +2125,11 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
       <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1924,8 +2147,11 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
       <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1943,8 +2169,11 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
       <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1962,8 +2191,11 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
       <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>